<commit_message>
Daily EOD data and reports for 2026-08-06
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260806.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260806.xlsx
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.29</v>
+        <v>2.31</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.05%</t>
+          <t>5.96%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>160300</v>
+        <v>161700</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>7700</v>
+        <v>9100</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.05</v>
+        <v>1.035</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.05</v>
+        <v>-0.065</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-4.55%</t>
+          <t>-5.91%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>60330.9</v>
+        <v>59469.03</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-2872.9</v>
+        <v>-3734.77</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>62.62</v>
+        <v>62.82</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.08</v>
+        <v>0.28</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>692890.3</v>
+        <v>695103.3</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>885.2</v>
+        <v>3098.2</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>178.77</v>
+        <v>179.87</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.54</v>
+        <v>1.64</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.30%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.855</v>
+        <v>0.845</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.91%</t>
+          <t>3.68%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>8550</v>
+        <v>8450</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>131.985</v>
+        <v>132.36</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1.325</v>
+        <v>1.7</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.01%</t>
+          <t>1.30%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>527940</v>
+        <v>529440</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>5300</v>
+        <v>6800</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.26</v>
+        <v>0.275</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-3.70%</t>
+          <t>1.85%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5200</v>
+        <v>5500</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-200</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.091</v>
+        <v>0.092</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>1.10%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>856.49</v>
+        <v>865.9</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>9.41</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.098</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.007</v>
+        <v>-0.005</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-6.67%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>588</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-42</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>38.56</v>
+        <v>38.53</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.08%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.795</v>
+        <v>31.72</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.015</v>
+        <v>-0.06</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.05%</t>
+          <t>-0.19%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>40951.96</v>
+        <v>40855.36</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>19.32</v>
+        <v>-77.28</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1722150.09</v>
+        <v>1726526.03</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>17448.67</v>
+        <v>21824.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>